<commit_message>
fix number digits and change columns to chinese
</commit_message>
<xml_diff>
--- a/Marini_iDigBio_306museums_coord_with_country_for518Map.xlsx
+++ b/Marini_iDigBio_306museums_coord_with_country_for518Map.xlsx
@@ -5,10 +5,10 @@
   <workbookPr defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Yiru Cheng\Dropbox\2022 Academia Sinica\Research\data\Egg\Global egg collection\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Yiru Cheng\Dropbox\2022 Academia Sinica\non-research\2026鳥蛋展覽\全球鳥蛋博物館地圖\antigravity\global-egg-dataset-main\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A5582A43-BE1C-4439-96F6-42404FD722BE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C9DEBE0F-4D95-4585-9FF0-0CAFC59988FB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-98" yWindow="-98" windowWidth="21795" windowHeight="12975" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -19,7 +19,7 @@
     <externalReference r:id="rId2"/>
   </externalReferences>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Sheet1!$A$1:$I$306</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Sheet1!$A$1:$I$307</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
@@ -3006,6 +3006,9 @@
 <file path=xl/externalLinks/externalLink1.xml><?xml version="1.0" encoding="utf-8"?>
 <externalLink xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xxl21="http://schemas.microsoft.com/office/spreadsheetml/2021/extlinks2021" mc:Ignorable="x14 xxl21">
   <externalBook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1">
+    <xxl21:alternateUrls>
+      <xxl21:relativeUrl r:id="rId2"/>
+    </xxl21:alternateUrls>
     <sheetNames>
       <sheetName val="Marini+iDigBio"/>
       <sheetName val="stats-211Museum"/>
@@ -9184,7 +9187,7 @@
         <v>659</v>
       </c>
     </row>
-    <row r="2" spans="1:10" ht="45" x14ac:dyDescent="0.45">
+    <row r="2" spans="1:10" x14ac:dyDescent="0.45">
       <c r="A2" t="s">
         <v>6</v>
       </c>
@@ -9283,7 +9286,7 @@
         <v>662</v>
       </c>
     </row>
-    <row r="5" spans="1:10" ht="75" x14ac:dyDescent="0.45">
+    <row r="5" spans="1:10" x14ac:dyDescent="0.45">
       <c r="A5" t="s">
         <v>9</v>
       </c>
@@ -9316,7 +9319,7 @@
         <v>663</v>
       </c>
     </row>
-    <row r="6" spans="1:10" ht="45" x14ac:dyDescent="0.45">
+    <row r="6" spans="1:10" x14ac:dyDescent="0.45">
       <c r="A6" t="s">
         <v>10</v>
       </c>
@@ -9349,7 +9352,7 @@
         <v>664</v>
       </c>
     </row>
-    <row r="7" spans="1:10" ht="45" x14ac:dyDescent="0.45">
+    <row r="7" spans="1:10" x14ac:dyDescent="0.45">
       <c r="A7" t="s">
         <v>11</v>
       </c>
@@ -9415,7 +9418,7 @@
         <v>666</v>
       </c>
     </row>
-    <row r="9" spans="1:10" ht="45" x14ac:dyDescent="0.45">
+    <row r="9" spans="1:10" ht="30" x14ac:dyDescent="0.45">
       <c r="A9" t="s">
         <v>13</v>
       </c>
@@ -9448,7 +9451,7 @@
         <v>667</v>
       </c>
     </row>
-    <row r="10" spans="1:10" ht="45" x14ac:dyDescent="0.45">
+    <row r="10" spans="1:10" x14ac:dyDescent="0.45">
       <c r="A10" t="s">
         <v>14</v>
       </c>
@@ -9481,7 +9484,7 @@
         <v>668</v>
       </c>
     </row>
-    <row r="11" spans="1:10" ht="30" x14ac:dyDescent="0.45">
+    <row r="11" spans="1:10" x14ac:dyDescent="0.45">
       <c r="A11" t="s">
         <v>15</v>
       </c>
@@ -9514,7 +9517,7 @@
         <v>669</v>
       </c>
     </row>
-    <row r="12" spans="1:10" ht="60" x14ac:dyDescent="0.45">
+    <row r="12" spans="1:10" x14ac:dyDescent="0.45">
       <c r="A12" t="s">
         <v>16</v>
       </c>
@@ -9578,7 +9581,7 @@
       </c>
       <c r="J13" s="12"/>
     </row>
-    <row r="14" spans="1:10" ht="75" x14ac:dyDescent="0.45">
+    <row r="14" spans="1:10" ht="30" x14ac:dyDescent="0.45">
       <c r="A14" t="s">
         <v>18</v>
       </c>
@@ -9611,7 +9614,7 @@
         <v>671</v>
       </c>
     </row>
-    <row r="15" spans="1:10" ht="45" x14ac:dyDescent="0.45">
+    <row r="15" spans="1:10" x14ac:dyDescent="0.45">
       <c r="A15" t="s">
         <v>19</v>
       </c>
@@ -9644,7 +9647,7 @@
         <v>672</v>
       </c>
     </row>
-    <row r="16" spans="1:10" ht="60" x14ac:dyDescent="0.45">
+    <row r="16" spans="1:10" ht="30" x14ac:dyDescent="0.45">
       <c r="A16" t="s">
         <v>20</v>
       </c>
@@ -9677,7 +9680,7 @@
         <v>673</v>
       </c>
     </row>
-    <row r="17" spans="1:10" ht="45" x14ac:dyDescent="0.45">
+    <row r="17" spans="1:10" ht="30" x14ac:dyDescent="0.45">
       <c r="A17" t="s">
         <v>21</v>
       </c>
@@ -9710,7 +9713,7 @@
         <v>674</v>
       </c>
     </row>
-    <row r="18" spans="1:10" ht="30" x14ac:dyDescent="0.45">
+    <row r="18" spans="1:10" x14ac:dyDescent="0.45">
       <c r="A18" t="s">
         <v>22</v>
       </c>
@@ -9743,7 +9746,7 @@
         <v>675</v>
       </c>
     </row>
-    <row r="19" spans="1:10" ht="60" x14ac:dyDescent="0.45">
+    <row r="19" spans="1:10" ht="30" x14ac:dyDescent="0.45">
       <c r="A19" t="s">
         <v>23</v>
       </c>
@@ -9776,7 +9779,7 @@
         <v>676</v>
       </c>
     </row>
-    <row r="20" spans="1:10" ht="30" x14ac:dyDescent="0.45">
+    <row r="20" spans="1:10" x14ac:dyDescent="0.45">
       <c r="A20" t="s">
         <v>24</v>
       </c>
@@ -9809,7 +9812,7 @@
         <v>677</v>
       </c>
     </row>
-    <row r="21" spans="1:10" ht="45" x14ac:dyDescent="0.45">
+    <row r="21" spans="1:10" ht="30" x14ac:dyDescent="0.45">
       <c r="A21" t="s">
         <v>25</v>
       </c>
@@ -9842,7 +9845,7 @@
         <v>678</v>
       </c>
     </row>
-    <row r="22" spans="1:10" ht="45" x14ac:dyDescent="0.45">
+    <row r="22" spans="1:10" ht="30" x14ac:dyDescent="0.45">
       <c r="A22" t="s">
         <v>26</v>
       </c>
@@ -9875,7 +9878,7 @@
         <v>679</v>
       </c>
     </row>
-    <row r="23" spans="1:10" ht="60" x14ac:dyDescent="0.45">
+    <row r="23" spans="1:10" x14ac:dyDescent="0.45">
       <c r="A23" t="s">
         <v>27</v>
       </c>
@@ -9908,7 +9911,7 @@
         <v>680</v>
       </c>
     </row>
-    <row r="24" spans="1:10" ht="45" x14ac:dyDescent="0.45">
+    <row r="24" spans="1:10" x14ac:dyDescent="0.45">
       <c r="A24" t="s">
         <v>28</v>
       </c>
@@ -9941,7 +9944,7 @@
         <v>681</v>
       </c>
     </row>
-    <row r="25" spans="1:10" ht="45" x14ac:dyDescent="0.45">
+    <row r="25" spans="1:10" ht="30" x14ac:dyDescent="0.45">
       <c r="A25" t="s">
         <v>29</v>
       </c>
@@ -9974,7 +9977,7 @@
         <v>682</v>
       </c>
     </row>
-    <row r="26" spans="1:10" ht="45" x14ac:dyDescent="0.45">
+    <row r="26" spans="1:10" x14ac:dyDescent="0.45">
       <c r="A26" t="s">
         <v>30</v>
       </c>
@@ -10007,7 +10010,7 @@
         <v>683</v>
       </c>
     </row>
-    <row r="27" spans="1:10" ht="90" x14ac:dyDescent="0.45">
+    <row r="27" spans="1:10" ht="30" x14ac:dyDescent="0.45">
       <c r="A27" t="s">
         <v>31</v>
       </c>
@@ -10040,7 +10043,7 @@
         <v>684</v>
       </c>
     </row>
-    <row r="28" spans="1:10" ht="120" x14ac:dyDescent="0.45">
+    <row r="28" spans="1:10" ht="30" x14ac:dyDescent="0.45">
       <c r="A28" t="s">
         <v>32</v>
       </c>
@@ -10073,7 +10076,7 @@
         <v>685</v>
       </c>
     </row>
-    <row r="29" spans="1:10" ht="45" x14ac:dyDescent="0.45">
+    <row r="29" spans="1:10" ht="30" x14ac:dyDescent="0.45">
       <c r="A29" t="s">
         <v>33</v>
       </c>
@@ -10106,7 +10109,7 @@
         <v>686</v>
       </c>
     </row>
-    <row r="30" spans="1:10" ht="75" x14ac:dyDescent="0.45">
+    <row r="30" spans="1:10" ht="30" x14ac:dyDescent="0.45">
       <c r="A30" t="s">
         <v>34</v>
       </c>
@@ -10139,7 +10142,7 @@
         <v>687</v>
       </c>
     </row>
-    <row r="31" spans="1:10" ht="45" x14ac:dyDescent="0.45">
+    <row r="31" spans="1:10" ht="30" x14ac:dyDescent="0.45">
       <c r="A31" t="s">
         <v>35</v>
       </c>
@@ -10172,7 +10175,7 @@
         <v>688</v>
       </c>
     </row>
-    <row r="32" spans="1:10" ht="60" x14ac:dyDescent="0.45">
+    <row r="32" spans="1:10" ht="30" x14ac:dyDescent="0.45">
       <c r="A32" t="s">
         <v>36</v>
       </c>
@@ -10205,7 +10208,7 @@
         <v>689</v>
       </c>
     </row>
-    <row r="33" spans="1:10" ht="45" x14ac:dyDescent="0.45">
+    <row r="33" spans="1:10" x14ac:dyDescent="0.45">
       <c r="A33" t="s">
         <v>37</v>
       </c>
@@ -10238,7 +10241,7 @@
         <v>690</v>
       </c>
     </row>
-    <row r="34" spans="1:10" ht="60" x14ac:dyDescent="0.45">
+    <row r="34" spans="1:10" ht="30" x14ac:dyDescent="0.45">
       <c r="A34" t="s">
         <v>38</v>
       </c>
@@ -10271,7 +10274,7 @@
         <v>691</v>
       </c>
     </row>
-    <row r="35" spans="1:10" ht="60" x14ac:dyDescent="0.45">
+    <row r="35" spans="1:10" ht="30" x14ac:dyDescent="0.45">
       <c r="A35" t="s">
         <v>39</v>
       </c>
@@ -10304,7 +10307,7 @@
         <v>692</v>
       </c>
     </row>
-    <row r="36" spans="1:10" ht="75" x14ac:dyDescent="0.45">
+    <row r="36" spans="1:10" ht="30" x14ac:dyDescent="0.45">
       <c r="A36" t="s">
         <v>40</v>
       </c>
@@ -10337,7 +10340,7 @@
         <v>693</v>
       </c>
     </row>
-    <row r="37" spans="1:10" ht="30" x14ac:dyDescent="0.45">
+    <row r="37" spans="1:10" x14ac:dyDescent="0.45">
       <c r="A37" t="s">
         <v>41</v>
       </c>
@@ -10370,7 +10373,7 @@
         <v>675</v>
       </c>
     </row>
-    <row r="38" spans="1:10" ht="45" x14ac:dyDescent="0.45">
+    <row r="38" spans="1:10" x14ac:dyDescent="0.45">
       <c r="A38" t="s">
         <v>42</v>
       </c>
@@ -10403,7 +10406,7 @@
         <v>694</v>
       </c>
     </row>
-    <row r="39" spans="1:10" ht="75" x14ac:dyDescent="0.45">
+    <row r="39" spans="1:10" ht="30" x14ac:dyDescent="0.45">
       <c r="A39" t="s">
         <v>43</v>
       </c>
@@ -10436,7 +10439,7 @@
         <v>695</v>
       </c>
     </row>
-    <row r="40" spans="1:10" ht="60" x14ac:dyDescent="0.45">
+    <row r="40" spans="1:10" x14ac:dyDescent="0.45">
       <c r="A40" t="s">
         <v>44</v>
       </c>
@@ -10469,7 +10472,7 @@
         <v>696</v>
       </c>
     </row>
-    <row r="41" spans="1:10" ht="75" x14ac:dyDescent="0.45">
+    <row r="41" spans="1:10" ht="30" x14ac:dyDescent="0.45">
       <c r="A41" t="s">
         <v>45</v>
       </c>
@@ -10502,7 +10505,7 @@
         <v>697</v>
       </c>
     </row>
-    <row r="42" spans="1:10" ht="45" x14ac:dyDescent="0.45">
+    <row r="42" spans="1:10" ht="30" x14ac:dyDescent="0.45">
       <c r="A42" t="s">
         <v>46</v>
       </c>
@@ -10535,7 +10538,7 @@
         <v>698</v>
       </c>
     </row>
-    <row r="43" spans="1:10" ht="90" x14ac:dyDescent="0.45">
+    <row r="43" spans="1:10" ht="30" x14ac:dyDescent="0.45">
       <c r="A43" t="s">
         <v>47</v>
       </c>
@@ -10568,7 +10571,7 @@
         <v>699</v>
       </c>
     </row>
-    <row r="44" spans="1:10" ht="45" x14ac:dyDescent="0.45">
+    <row r="44" spans="1:10" ht="30" x14ac:dyDescent="0.45">
       <c r="A44" t="s">
         <v>48</v>
       </c>
@@ -10601,7 +10604,7 @@
         <v>700</v>
       </c>
     </row>
-    <row r="45" spans="1:10" ht="45" x14ac:dyDescent="0.45">
+    <row r="45" spans="1:10" x14ac:dyDescent="0.45">
       <c r="A45" t="s">
         <v>49</v>
       </c>
@@ -10634,7 +10637,7 @@
         <v>701</v>
       </c>
     </row>
-    <row r="46" spans="1:10" ht="45" x14ac:dyDescent="0.45">
+    <row r="46" spans="1:10" ht="30" x14ac:dyDescent="0.45">
       <c r="A46" t="s">
         <v>50</v>
       </c>
@@ -10667,7 +10670,7 @@
         <v>702</v>
       </c>
     </row>
-    <row r="47" spans="1:10" ht="30" x14ac:dyDescent="0.45">
+    <row r="47" spans="1:10" x14ac:dyDescent="0.45">
       <c r="A47" t="s">
         <v>24</v>
       </c>
@@ -10700,7 +10703,7 @@
         <v>677</v>
       </c>
     </row>
-    <row r="48" spans="1:10" ht="30" x14ac:dyDescent="0.45">
+    <row r="48" spans="1:10" x14ac:dyDescent="0.45">
       <c r="A48" t="s">
         <v>41</v>
       </c>
@@ -10733,7 +10736,7 @@
         <v>675</v>
       </c>
     </row>
-    <row r="49" spans="1:10" ht="45" x14ac:dyDescent="0.45">
+    <row r="49" spans="1:10" x14ac:dyDescent="0.45">
       <c r="A49" t="s">
         <v>51</v>
       </c>
@@ -10766,7 +10769,7 @@
         <v>703</v>
       </c>
     </row>
-    <row r="50" spans="1:10" ht="60" x14ac:dyDescent="0.45">
+    <row r="50" spans="1:10" x14ac:dyDescent="0.45">
       <c r="A50" t="s">
         <v>52</v>
       </c>
@@ -10799,7 +10802,7 @@
         <v>704</v>
       </c>
     </row>
-    <row r="51" spans="1:10" ht="60" x14ac:dyDescent="0.45">
+    <row r="51" spans="1:10" ht="30" x14ac:dyDescent="0.45">
       <c r="A51" t="s">
         <v>53</v>
       </c>
@@ -10832,7 +10835,7 @@
         <v>705</v>
       </c>
     </row>
-    <row r="52" spans="1:10" ht="45" x14ac:dyDescent="0.45">
+    <row r="52" spans="1:10" ht="30" x14ac:dyDescent="0.45">
       <c r="A52" t="s">
         <v>54</v>
       </c>
@@ -10865,7 +10868,7 @@
         <v>706</v>
       </c>
     </row>
-    <row r="53" spans="1:10" ht="60" x14ac:dyDescent="0.45">
+    <row r="53" spans="1:10" x14ac:dyDescent="0.45">
       <c r="A53" t="s">
         <v>55</v>
       </c>
@@ -10929,7 +10932,7 @@
       </c>
       <c r="J54" s="12"/>
     </row>
-    <row r="55" spans="1:10" ht="60" x14ac:dyDescent="0.45">
+    <row r="55" spans="1:10" x14ac:dyDescent="0.45">
       <c r="A55" t="s">
         <v>57</v>
       </c>
@@ -10962,7 +10965,7 @@
         <v>708</v>
       </c>
     </row>
-    <row r="56" spans="1:10" ht="60" x14ac:dyDescent="0.45">
+    <row r="56" spans="1:10" x14ac:dyDescent="0.45">
       <c r="A56" t="s">
         <v>58</v>
       </c>
@@ -10995,7 +10998,7 @@
         <v>709</v>
       </c>
     </row>
-    <row r="57" spans="1:10" ht="30" x14ac:dyDescent="0.45">
+    <row r="57" spans="1:10" x14ac:dyDescent="0.45">
       <c r="A57" t="s">
         <v>24</v>
       </c>
@@ -11028,7 +11031,7 @@
         <v>677</v>
       </c>
     </row>
-    <row r="58" spans="1:10" ht="45" x14ac:dyDescent="0.45">
+    <row r="58" spans="1:10" x14ac:dyDescent="0.45">
       <c r="A58" t="s">
         <v>59</v>
       </c>
@@ -11061,7 +11064,7 @@
         <v>710</v>
       </c>
     </row>
-    <row r="59" spans="1:10" ht="60" x14ac:dyDescent="0.45">
+    <row r="59" spans="1:10" x14ac:dyDescent="0.45">
       <c r="A59" t="s">
         <v>60</v>
       </c>
@@ -11094,7 +11097,7 @@
         <v>711</v>
       </c>
     </row>
-    <row r="60" spans="1:10" ht="45" x14ac:dyDescent="0.45">
+    <row r="60" spans="1:10" x14ac:dyDescent="0.45">
       <c r="A60" t="s">
         <v>61</v>
       </c>
@@ -11127,7 +11130,7 @@
         <v>712</v>
       </c>
     </row>
-    <row r="61" spans="1:10" ht="45" x14ac:dyDescent="0.45">
+    <row r="61" spans="1:10" x14ac:dyDescent="0.45">
       <c r="A61" t="s">
         <v>62</v>
       </c>
@@ -11160,7 +11163,7 @@
         <v>713</v>
       </c>
     </row>
-    <row r="62" spans="1:10" ht="45" x14ac:dyDescent="0.45">
+    <row r="62" spans="1:10" x14ac:dyDescent="0.45">
       <c r="A62" t="s">
         <v>63</v>
       </c>
@@ -11193,7 +11196,7 @@
         <v>714</v>
       </c>
     </row>
-    <row r="63" spans="1:10" ht="75" x14ac:dyDescent="0.45">
+    <row r="63" spans="1:10" ht="30" x14ac:dyDescent="0.45">
       <c r="A63" t="s">
         <v>64</v>
       </c>
@@ -11226,7 +11229,7 @@
         <v>715</v>
       </c>
     </row>
-    <row r="64" spans="1:10" ht="45" x14ac:dyDescent="0.45">
+    <row r="64" spans="1:10" ht="30" x14ac:dyDescent="0.45">
       <c r="A64" t="s">
         <v>65</v>
       </c>
@@ -11259,7 +11262,7 @@
         <v>679</v>
       </c>
     </row>
-    <row r="65" spans="1:10" ht="30" x14ac:dyDescent="0.45">
+    <row r="65" spans="1:10" x14ac:dyDescent="0.45">
       <c r="A65" t="s">
         <v>66</v>
       </c>
@@ -11292,7 +11295,7 @@
         <v>716</v>
       </c>
     </row>
-    <row r="66" spans="1:10" ht="30" x14ac:dyDescent="0.45">
+    <row r="66" spans="1:10" x14ac:dyDescent="0.45">
       <c r="A66" t="s">
         <v>67</v>
       </c>
@@ -11325,7 +11328,7 @@
         <v>717</v>
       </c>
     </row>
-    <row r="67" spans="1:10" ht="45" x14ac:dyDescent="0.45">
+    <row r="67" spans="1:10" x14ac:dyDescent="0.45">
       <c r="A67" t="s">
         <v>68</v>
       </c>
@@ -11358,7 +11361,7 @@
         <v>665</v>
       </c>
     </row>
-    <row r="68" spans="1:10" ht="60" x14ac:dyDescent="0.45">
+    <row r="68" spans="1:10" x14ac:dyDescent="0.45">
       <c r="A68" t="s">
         <v>69</v>
       </c>
@@ -11391,7 +11394,7 @@
         <v>718</v>
       </c>
     </row>
-    <row r="69" spans="1:10" ht="180" x14ac:dyDescent="0.45">
+    <row r="69" spans="1:10" ht="60" x14ac:dyDescent="0.45">
       <c r="A69" t="s">
         <v>70</v>
       </c>
@@ -11424,7 +11427,7 @@
         <v>719</v>
       </c>
     </row>
-    <row r="70" spans="1:10" ht="75" x14ac:dyDescent="0.45">
+    <row r="70" spans="1:10" ht="30" x14ac:dyDescent="0.45">
       <c r="A70" t="s">
         <v>71</v>
       </c>
@@ -11457,7 +11460,7 @@
         <v>720</v>
       </c>
     </row>
-    <row r="71" spans="1:10" ht="45" x14ac:dyDescent="0.45">
+    <row r="71" spans="1:10" ht="30" x14ac:dyDescent="0.45">
       <c r="A71" t="s">
         <v>72</v>
       </c>
@@ -11490,7 +11493,7 @@
         <v>721</v>
       </c>
     </row>
-    <row r="72" spans="1:10" ht="45" x14ac:dyDescent="0.45">
+    <row r="72" spans="1:10" ht="30" x14ac:dyDescent="0.45">
       <c r="A72" t="s">
         <v>73</v>
       </c>
@@ -11523,7 +11526,7 @@
         <v>722</v>
       </c>
     </row>
-    <row r="73" spans="1:10" ht="75" x14ac:dyDescent="0.45">
+    <row r="73" spans="1:10" ht="30" x14ac:dyDescent="0.45">
       <c r="A73" t="s">
         <v>74</v>
       </c>
@@ -11556,7 +11559,7 @@
         <v>723</v>
       </c>
     </row>
-    <row r="74" spans="1:10" ht="60" x14ac:dyDescent="0.45">
+    <row r="74" spans="1:10" ht="30" x14ac:dyDescent="0.45">
       <c r="A74" t="s">
         <v>75</v>
       </c>
@@ -11589,7 +11592,7 @@
         <v>724</v>
       </c>
     </row>
-    <row r="75" spans="1:10" ht="60" x14ac:dyDescent="0.45">
+    <row r="75" spans="1:10" ht="30" x14ac:dyDescent="0.45">
       <c r="A75" t="s">
         <v>76</v>
       </c>
@@ -11622,7 +11625,7 @@
         <v>725</v>
       </c>
     </row>
-    <row r="76" spans="1:10" ht="75" x14ac:dyDescent="0.45">
+    <row r="76" spans="1:10" ht="30" x14ac:dyDescent="0.45">
       <c r="A76" t="s">
         <v>77</v>
       </c>
@@ -11655,7 +11658,7 @@
         <v>726</v>
       </c>
     </row>
-    <row r="77" spans="1:10" ht="45" x14ac:dyDescent="0.45">
+    <row r="77" spans="1:10" ht="30" x14ac:dyDescent="0.45">
       <c r="A77" t="s">
         <v>78</v>
       </c>
@@ -11688,7 +11691,7 @@
         <v>727</v>
       </c>
     </row>
-    <row r="78" spans="1:10" ht="105" x14ac:dyDescent="0.45">
+    <row r="78" spans="1:10" ht="30" x14ac:dyDescent="0.45">
       <c r="A78" t="s">
         <v>79</v>
       </c>
@@ -11711,8 +11714,7 @@
         <v>448</v>
       </c>
       <c r="H78" s="6">
-        <f>VLOOKUP(A78, '[1]Marini+iDigBio'!$D$2:$J$306, 7, FALSE)</f>
-        <v>4396.666666666667</v>
+        <v>23288</v>
       </c>
       <c r="I78">
         <v>1</v>
@@ -11721,7 +11723,7 @@
         <v>728</v>
       </c>
     </row>
-    <row r="79" spans="1:10" ht="45" x14ac:dyDescent="0.45">
+    <row r="79" spans="1:10" ht="30" x14ac:dyDescent="0.45">
       <c r="A79" t="s">
         <v>80</v>
       </c>
@@ -11754,7 +11756,7 @@
         <v>729</v>
       </c>
     </row>
-    <row r="80" spans="1:10" ht="45" x14ac:dyDescent="0.45">
+    <row r="80" spans="1:10" x14ac:dyDescent="0.45">
       <c r="A80" t="s">
         <v>81</v>
       </c>
@@ -11787,7 +11789,7 @@
         <v>730</v>
       </c>
     </row>
-    <row r="81" spans="1:10" ht="45" x14ac:dyDescent="0.45">
+    <row r="81" spans="1:10" x14ac:dyDescent="0.45">
       <c r="A81" t="s">
         <v>82</v>
       </c>
@@ -11851,7 +11853,7 @@
       </c>
       <c r="J82" s="12"/>
     </row>
-    <row r="83" spans="1:10" ht="60" x14ac:dyDescent="0.45">
+    <row r="83" spans="1:10" x14ac:dyDescent="0.45">
       <c r="A83" t="s">
         <v>84</v>
       </c>
@@ -11884,7 +11886,7 @@
         <v>732</v>
       </c>
     </row>
-    <row r="84" spans="1:10" ht="60" x14ac:dyDescent="0.45">
+    <row r="84" spans="1:10" ht="45" x14ac:dyDescent="0.45">
       <c r="A84" t="s">
         <v>85</v>
       </c>
@@ -11917,7 +11919,7 @@
         <v>733</v>
       </c>
     </row>
-    <row r="85" spans="1:10" ht="45" x14ac:dyDescent="0.45">
+    <row r="85" spans="1:10" ht="30" x14ac:dyDescent="0.45">
       <c r="A85" t="s">
         <v>86</v>
       </c>
@@ -11950,7 +11952,7 @@
         <v>734</v>
       </c>
     </row>
-    <row r="86" spans="1:10" ht="45" x14ac:dyDescent="0.45">
+    <row r="86" spans="1:10" x14ac:dyDescent="0.45">
       <c r="A86" t="s">
         <v>87</v>
       </c>
@@ -11983,7 +11985,7 @@
         <v>735</v>
       </c>
     </row>
-    <row r="87" spans="1:10" ht="60" x14ac:dyDescent="0.45">
+    <row r="87" spans="1:10" x14ac:dyDescent="0.45">
       <c r="A87" t="s">
         <v>88</v>
       </c>
@@ -12016,7 +12018,7 @@
         <v>736</v>
       </c>
     </row>
-    <row r="88" spans="1:10" ht="75" x14ac:dyDescent="0.45">
+    <row r="88" spans="1:10" x14ac:dyDescent="0.45">
       <c r="A88" t="s">
         <v>89</v>
       </c>
@@ -12049,7 +12051,7 @@
         <v>737</v>
       </c>
     </row>
-    <row r="89" spans="1:10" ht="45" x14ac:dyDescent="0.45">
+    <row r="89" spans="1:10" x14ac:dyDescent="0.45">
       <c r="A89" t="s">
         <v>90</v>
       </c>
@@ -12082,7 +12084,7 @@
         <v>738</v>
       </c>
     </row>
-    <row r="90" spans="1:10" ht="60" x14ac:dyDescent="0.45">
+    <row r="90" spans="1:10" x14ac:dyDescent="0.45">
       <c r="A90" t="s">
         <v>91</v>
       </c>
@@ -12115,7 +12117,7 @@
         <v>739</v>
       </c>
     </row>
-    <row r="91" spans="1:10" ht="45" x14ac:dyDescent="0.45">
+    <row r="91" spans="1:10" x14ac:dyDescent="0.45">
       <c r="A91" t="s">
         <v>92</v>
       </c>
@@ -12148,7 +12150,7 @@
         <v>740</v>
       </c>
     </row>
-    <row r="92" spans="1:10" ht="75" x14ac:dyDescent="0.45">
+    <row r="92" spans="1:10" ht="30" x14ac:dyDescent="0.45">
       <c r="A92" t="s">
         <v>93</v>
       </c>
@@ -12181,7 +12183,7 @@
         <v>741</v>
       </c>
     </row>
-    <row r="93" spans="1:10" ht="75" x14ac:dyDescent="0.45">
+    <row r="93" spans="1:10" ht="30" x14ac:dyDescent="0.45">
       <c r="A93" t="s">
         <v>94</v>
       </c>
@@ -12247,7 +12249,7 @@
         <v>743</v>
       </c>
     </row>
-    <row r="95" spans="1:10" ht="45" x14ac:dyDescent="0.45">
+    <row r="95" spans="1:10" x14ac:dyDescent="0.45">
       <c r="A95" t="s">
         <v>96</v>
       </c>
@@ -12280,7 +12282,7 @@
         <v>744</v>
       </c>
     </row>
-    <row r="96" spans="1:10" ht="45" x14ac:dyDescent="0.45">
+    <row r="96" spans="1:10" x14ac:dyDescent="0.45">
       <c r="A96" t="s">
         <v>97</v>
       </c>
@@ -12313,7 +12315,7 @@
         <v>745</v>
       </c>
     </row>
-    <row r="97" spans="1:10" ht="60" x14ac:dyDescent="0.45">
+    <row r="97" spans="1:10" ht="30" x14ac:dyDescent="0.45">
       <c r="A97" t="s">
         <v>98</v>
       </c>
@@ -12346,7 +12348,7 @@
         <v>746</v>
       </c>
     </row>
-    <row r="98" spans="1:10" ht="60" x14ac:dyDescent="0.45">
+    <row r="98" spans="1:10" ht="30" x14ac:dyDescent="0.45">
       <c r="A98" t="s">
         <v>99</v>
       </c>
@@ -12412,7 +12414,7 @@
         <v>748</v>
       </c>
     </row>
-    <row r="100" spans="1:10" ht="30" x14ac:dyDescent="0.45">
+    <row r="100" spans="1:10" x14ac:dyDescent="0.45">
       <c r="A100" t="s">
         <v>24</v>
       </c>
@@ -12445,7 +12447,7 @@
         <v>677</v>
       </c>
     </row>
-    <row r="101" spans="1:10" ht="45" x14ac:dyDescent="0.45">
+    <row r="101" spans="1:10" x14ac:dyDescent="0.45">
       <c r="A101" t="s">
         <v>101</v>
       </c>
@@ -12478,7 +12480,7 @@
         <v>749</v>
       </c>
     </row>
-    <row r="102" spans="1:10" ht="45" x14ac:dyDescent="0.45">
+    <row r="102" spans="1:10" x14ac:dyDescent="0.45">
       <c r="A102" t="s">
         <v>102</v>
       </c>
@@ -12511,7 +12513,7 @@
         <v>750</v>
       </c>
     </row>
-    <row r="103" spans="1:10" ht="60" x14ac:dyDescent="0.45">
+    <row r="103" spans="1:10" x14ac:dyDescent="0.45">
       <c r="A103" t="s">
         <v>103</v>
       </c>
@@ -12575,7 +12577,7 @@
       </c>
       <c r="J104" s="12"/>
     </row>
-    <row r="105" spans="1:10" ht="45" x14ac:dyDescent="0.45">
+    <row r="105" spans="1:10" ht="30" x14ac:dyDescent="0.45">
       <c r="A105" t="s">
         <v>105</v>
       </c>
@@ -12608,7 +12610,7 @@
         <v>679</v>
       </c>
     </row>
-    <row r="106" spans="1:10" ht="45" x14ac:dyDescent="0.45">
+    <row r="106" spans="1:10" x14ac:dyDescent="0.45">
       <c r="A106" t="s">
         <v>106</v>
       </c>
@@ -12641,7 +12643,7 @@
         <v>752</v>
       </c>
     </row>
-    <row r="107" spans="1:10" ht="30" x14ac:dyDescent="0.45">
+    <row r="107" spans="1:10" x14ac:dyDescent="0.45">
       <c r="A107" t="s">
         <v>107</v>
       </c>
@@ -12674,7 +12676,7 @@
         <v>753</v>
       </c>
     </row>
-    <row r="108" spans="1:10" ht="60" x14ac:dyDescent="0.45">
+    <row r="108" spans="1:10" ht="30" x14ac:dyDescent="0.45">
       <c r="A108" t="s">
         <v>108</v>
       </c>
@@ -12707,7 +12709,7 @@
         <v>754</v>
       </c>
     </row>
-    <row r="109" spans="1:10" ht="120" x14ac:dyDescent="0.45">
+    <row r="109" spans="1:10" ht="45" x14ac:dyDescent="0.45">
       <c r="A109" t="s">
         <v>109</v>
       </c>
@@ -12740,7 +12742,7 @@
         <v>755</v>
       </c>
     </row>
-    <row r="110" spans="1:10" ht="45" x14ac:dyDescent="0.45">
+    <row r="110" spans="1:10" x14ac:dyDescent="0.45">
       <c r="A110" t="s">
         <v>110</v>
       </c>
@@ -12773,7 +12775,7 @@
         <v>756</v>
       </c>
     </row>
-    <row r="111" spans="1:10" ht="45" x14ac:dyDescent="0.45">
+    <row r="111" spans="1:10" x14ac:dyDescent="0.45">
       <c r="A111" t="s">
         <v>111</v>
       </c>
@@ -12839,7 +12841,7 @@
         <v>758</v>
       </c>
     </row>
-    <row r="113" spans="1:10" ht="60" x14ac:dyDescent="0.45">
+    <row r="113" spans="1:10" ht="30" x14ac:dyDescent="0.45">
       <c r="A113" t="s">
         <v>113</v>
       </c>
@@ -12872,7 +12874,7 @@
         <v>759</v>
       </c>
     </row>
-    <row r="114" spans="1:10" ht="45" x14ac:dyDescent="0.45">
+    <row r="114" spans="1:10" ht="30" x14ac:dyDescent="0.45">
       <c r="A114" t="s">
         <v>114</v>
       </c>
@@ -12905,7 +12907,7 @@
         <v>760</v>
       </c>
     </row>
-    <row r="115" spans="1:10" ht="105" x14ac:dyDescent="0.45">
+    <row r="115" spans="1:10" ht="30" x14ac:dyDescent="0.45">
       <c r="A115" t="s">
         <v>115</v>
       </c>
@@ -12969,7 +12971,7 @@
       </c>
       <c r="J116" s="12"/>
     </row>
-    <row r="117" spans="1:10" ht="45" x14ac:dyDescent="0.45">
+    <row r="117" spans="1:10" ht="30" x14ac:dyDescent="0.45">
       <c r="A117" t="s">
         <v>117</v>
       </c>
@@ -13002,7 +13004,7 @@
         <v>762</v>
       </c>
     </row>
-    <row r="118" spans="1:10" ht="75" x14ac:dyDescent="0.45">
+    <row r="118" spans="1:10" ht="30" x14ac:dyDescent="0.45">
       <c r="A118" t="s">
         <v>118</v>
       </c>
@@ -13035,7 +13037,7 @@
         <v>763</v>
       </c>
     </row>
-    <row r="119" spans="1:10" ht="45" x14ac:dyDescent="0.45">
+    <row r="119" spans="1:10" ht="30" x14ac:dyDescent="0.45">
       <c r="A119" t="s">
         <v>119</v>
       </c>
@@ -13068,7 +13070,7 @@
         <v>764</v>
       </c>
     </row>
-    <row r="120" spans="1:10" ht="45" x14ac:dyDescent="0.45">
+    <row r="120" spans="1:10" x14ac:dyDescent="0.45">
       <c r="A120" t="s">
         <v>120</v>
       </c>
@@ -13101,7 +13103,7 @@
         <v>765</v>
       </c>
     </row>
-    <row r="121" spans="1:10" ht="75" x14ac:dyDescent="0.45">
+    <row r="121" spans="1:10" ht="30" x14ac:dyDescent="0.45">
       <c r="A121" t="s">
         <v>121</v>
       </c>
@@ -13134,7 +13136,7 @@
         <v>766</v>
       </c>
     </row>
-    <row r="122" spans="1:10" ht="60" x14ac:dyDescent="0.45">
+    <row r="122" spans="1:10" ht="30" x14ac:dyDescent="0.45">
       <c r="A122" t="s">
         <v>122</v>
       </c>
@@ -13167,7 +13169,7 @@
         <v>767</v>
       </c>
     </row>
-    <row r="123" spans="1:10" ht="60" x14ac:dyDescent="0.45">
+    <row r="123" spans="1:10" x14ac:dyDescent="0.45">
       <c r="A123" t="s">
         <v>123</v>
       </c>
@@ -13200,7 +13202,7 @@
         <v>768</v>
       </c>
     </row>
-    <row r="124" spans="1:10" ht="60" x14ac:dyDescent="0.45">
+    <row r="124" spans="1:10" ht="30" x14ac:dyDescent="0.45">
       <c r="A124" t="s">
         <v>124</v>
       </c>
@@ -13233,7 +13235,7 @@
         <v>769</v>
       </c>
     </row>
-    <row r="125" spans="1:10" ht="45" x14ac:dyDescent="0.45">
+    <row r="125" spans="1:10" x14ac:dyDescent="0.45">
       <c r="A125" t="s">
         <v>125</v>
       </c>
@@ -13266,7 +13268,7 @@
         <v>770</v>
       </c>
     </row>
-    <row r="126" spans="1:10" ht="45" x14ac:dyDescent="0.45">
+    <row r="126" spans="1:10" x14ac:dyDescent="0.45">
       <c r="A126" t="s">
         <v>126</v>
       </c>
@@ -13299,7 +13301,7 @@
         <v>771</v>
       </c>
     </row>
-    <row r="127" spans="1:10" ht="60" x14ac:dyDescent="0.45">
+    <row r="127" spans="1:10" x14ac:dyDescent="0.45">
       <c r="A127" t="s">
         <v>127</v>
       </c>
@@ -13332,7 +13334,7 @@
         <v>772</v>
       </c>
     </row>
-    <row r="128" spans="1:10" ht="60" x14ac:dyDescent="0.45">
+    <row r="128" spans="1:10" x14ac:dyDescent="0.45">
       <c r="A128" t="s">
         <v>128</v>
       </c>
@@ -13365,7 +13367,7 @@
         <v>773</v>
       </c>
     </row>
-    <row r="129" spans="1:10" ht="45" x14ac:dyDescent="0.45">
+    <row r="129" spans="1:10" ht="30" x14ac:dyDescent="0.45">
       <c r="A129" t="s">
         <v>129</v>
       </c>
@@ -13431,7 +13433,7 @@
         <v>775</v>
       </c>
     </row>
-    <row r="131" spans="1:10" ht="60" x14ac:dyDescent="0.45">
+    <row r="131" spans="1:10" ht="30" x14ac:dyDescent="0.45">
       <c r="A131" t="s">
         <v>131</v>
       </c>
@@ -13464,7 +13466,7 @@
         <v>776</v>
       </c>
     </row>
-    <row r="132" spans="1:10" ht="60" x14ac:dyDescent="0.45">
+    <row r="132" spans="1:10" ht="30" x14ac:dyDescent="0.45">
       <c r="A132" t="s">
         <v>132</v>
       </c>
@@ -13530,7 +13532,7 @@
         <v>778</v>
       </c>
     </row>
-    <row r="134" spans="1:10" ht="60" x14ac:dyDescent="0.45">
+    <row r="134" spans="1:10" ht="45" x14ac:dyDescent="0.45">
       <c r="A134" t="s">
         <v>134</v>
       </c>
@@ -13563,7 +13565,7 @@
         <v>779</v>
       </c>
     </row>
-    <row r="135" spans="1:10" ht="60" x14ac:dyDescent="0.45">
+    <row r="135" spans="1:10" ht="30" x14ac:dyDescent="0.45">
       <c r="A135" t="s">
         <v>135</v>
       </c>
@@ -13596,7 +13598,7 @@
         <v>780</v>
       </c>
     </row>
-    <row r="136" spans="1:10" ht="45" x14ac:dyDescent="0.45">
+    <row r="136" spans="1:10" ht="30" x14ac:dyDescent="0.45">
       <c r="A136" t="s">
         <v>136</v>
       </c>
@@ -13629,7 +13631,7 @@
         <v>781</v>
       </c>
     </row>
-    <row r="137" spans="1:10" ht="60" x14ac:dyDescent="0.45">
+    <row r="137" spans="1:10" ht="30" x14ac:dyDescent="0.45">
       <c r="A137" t="s">
         <v>9</v>
       </c>
@@ -13662,7 +13664,7 @@
         <v>692</v>
       </c>
     </row>
-    <row r="138" spans="1:10" ht="45" x14ac:dyDescent="0.45">
+    <row r="138" spans="1:10" x14ac:dyDescent="0.45">
       <c r="A138" t="s">
         <v>137</v>
       </c>
@@ -13695,7 +13697,7 @@
         <v>782</v>
       </c>
     </row>
-    <row r="139" spans="1:10" ht="60" x14ac:dyDescent="0.45">
+    <row r="139" spans="1:10" x14ac:dyDescent="0.45">
       <c r="A139" t="s">
         <v>138</v>
       </c>
@@ -13728,7 +13730,7 @@
         <v>783</v>
       </c>
     </row>
-    <row r="140" spans="1:10" ht="45" x14ac:dyDescent="0.45">
+    <row r="140" spans="1:10" x14ac:dyDescent="0.45">
       <c r="A140" t="s">
         <v>139</v>
       </c>
@@ -13761,7 +13763,7 @@
         <v>784</v>
       </c>
     </row>
-    <row r="141" spans="1:10" ht="75" x14ac:dyDescent="0.45">
+    <row r="141" spans="1:10" ht="30" x14ac:dyDescent="0.45">
       <c r="A141" t="s">
         <v>9</v>
       </c>
@@ -13794,7 +13796,7 @@
         <v>785</v>
       </c>
     </row>
-    <row r="142" spans="1:10" ht="75" x14ac:dyDescent="0.45">
+    <row r="142" spans="1:10" x14ac:dyDescent="0.45">
       <c r="A142" t="s">
         <v>140</v>
       </c>
@@ -13860,7 +13862,7 @@
         <v>787</v>
       </c>
     </row>
-    <row r="144" spans="1:10" ht="45" x14ac:dyDescent="0.45">
+    <row r="144" spans="1:10" x14ac:dyDescent="0.45">
       <c r="A144" t="s">
         <v>142</v>
       </c>
@@ -13893,7 +13895,7 @@
         <v>788</v>
       </c>
     </row>
-    <row r="145" spans="1:10" ht="45" x14ac:dyDescent="0.45">
+    <row r="145" spans="1:10" ht="30" x14ac:dyDescent="0.45">
       <c r="A145" t="s">
         <v>13</v>
       </c>
@@ -13926,7 +13928,7 @@
         <v>667</v>
       </c>
     </row>
-    <row r="146" spans="1:10" ht="45" x14ac:dyDescent="0.45">
+    <row r="146" spans="1:10" x14ac:dyDescent="0.45">
       <c r="A146" t="s">
         <v>143</v>
       </c>
@@ -13959,7 +13961,7 @@
         <v>789</v>
       </c>
     </row>
-    <row r="147" spans="1:10" ht="60" x14ac:dyDescent="0.45">
+    <row r="147" spans="1:10" x14ac:dyDescent="0.45">
       <c r="A147" t="s">
         <v>144</v>
       </c>
@@ -13992,7 +13994,7 @@
         <v>790</v>
       </c>
     </row>
-    <row r="148" spans="1:10" ht="60" x14ac:dyDescent="0.45">
+    <row r="148" spans="1:10" ht="30" x14ac:dyDescent="0.45">
       <c r="A148" t="s">
         <v>145</v>
       </c>
@@ -14025,7 +14027,7 @@
         <v>791</v>
       </c>
     </row>
-    <row r="149" spans="1:10" ht="45" x14ac:dyDescent="0.45">
+    <row r="149" spans="1:10" ht="30" x14ac:dyDescent="0.45">
       <c r="A149" t="s">
         <v>146</v>
       </c>
@@ -14091,7 +14093,7 @@
         <v>793</v>
       </c>
     </row>
-    <row r="151" spans="1:10" ht="45" x14ac:dyDescent="0.45">
+    <row r="151" spans="1:10" x14ac:dyDescent="0.45">
       <c r="A151" t="s">
         <v>148</v>
       </c>
@@ -14124,7 +14126,7 @@
         <v>794</v>
       </c>
     </row>
-    <row r="152" spans="1:10" ht="75" x14ac:dyDescent="0.45">
+    <row r="152" spans="1:10" x14ac:dyDescent="0.45">
       <c r="A152" t="s">
         <v>149</v>
       </c>
@@ -14188,7 +14190,7 @@
       </c>
       <c r="J153" s="12"/>
     </row>
-    <row r="154" spans="1:10" ht="60" x14ac:dyDescent="0.45">
+    <row r="154" spans="1:10" ht="30" x14ac:dyDescent="0.45">
       <c r="A154" t="s">
         <v>151</v>
       </c>
@@ -14221,7 +14223,7 @@
         <v>796</v>
       </c>
     </row>
-    <row r="155" spans="1:10" ht="60" x14ac:dyDescent="0.45">
+    <row r="155" spans="1:10" x14ac:dyDescent="0.45">
       <c r="A155" t="s">
         <v>152</v>
       </c>
@@ -14254,7 +14256,7 @@
         <v>797</v>
       </c>
     </row>
-    <row r="156" spans="1:10" ht="60" x14ac:dyDescent="0.45">
+    <row r="156" spans="1:10" x14ac:dyDescent="0.45">
       <c r="A156" t="s">
         <v>153</v>
       </c>
@@ -14287,7 +14289,7 @@
         <v>798</v>
       </c>
     </row>
-    <row r="157" spans="1:10" ht="60" x14ac:dyDescent="0.45">
+    <row r="157" spans="1:10" ht="30" x14ac:dyDescent="0.45">
       <c r="A157" t="s">
         <v>154</v>
       </c>
@@ -14320,7 +14322,7 @@
         <v>799</v>
       </c>
     </row>
-    <row r="158" spans="1:10" ht="45" x14ac:dyDescent="0.45">
+    <row r="158" spans="1:10" ht="30" x14ac:dyDescent="0.45">
       <c r="A158" t="s">
         <v>155</v>
       </c>
@@ -14353,7 +14355,7 @@
         <v>800</v>
       </c>
     </row>
-    <row r="159" spans="1:10" ht="60" x14ac:dyDescent="0.45">
+    <row r="159" spans="1:10" x14ac:dyDescent="0.45">
       <c r="A159" t="s">
         <v>156</v>
       </c>
@@ -14386,7 +14388,7 @@
         <v>801</v>
       </c>
     </row>
-    <row r="160" spans="1:10" ht="45" x14ac:dyDescent="0.45">
+    <row r="160" spans="1:10" ht="30" x14ac:dyDescent="0.45">
       <c r="A160" t="s">
         <v>157</v>
       </c>
@@ -14419,7 +14421,7 @@
         <v>802</v>
       </c>
     </row>
-    <row r="161" spans="1:10" ht="75" x14ac:dyDescent="0.45">
+    <row r="161" spans="1:10" ht="30" x14ac:dyDescent="0.45">
       <c r="A161" t="s">
         <v>158</v>
       </c>
@@ -14452,7 +14454,7 @@
         <v>803</v>
       </c>
     </row>
-    <row r="162" spans="1:10" ht="75" x14ac:dyDescent="0.45">
+    <row r="162" spans="1:10" ht="30" x14ac:dyDescent="0.45">
       <c r="A162" t="s">
         <v>159</v>
       </c>
@@ -14485,7 +14487,7 @@
         <v>804</v>
       </c>
     </row>
-    <row r="163" spans="1:10" ht="60" x14ac:dyDescent="0.45">
+    <row r="163" spans="1:10" ht="30" x14ac:dyDescent="0.45">
       <c r="A163" t="s">
         <v>160</v>
       </c>
@@ -14549,7 +14551,7 @@
       </c>
       <c r="J164" s="12"/>
     </row>
-    <row r="165" spans="1:10" ht="45" x14ac:dyDescent="0.45">
+    <row r="165" spans="1:10" ht="30" x14ac:dyDescent="0.45">
       <c r="A165" t="s">
         <v>162</v>
       </c>
@@ -14582,7 +14584,7 @@
         <v>806</v>
       </c>
     </row>
-    <row r="166" spans="1:10" ht="60" x14ac:dyDescent="0.45">
+    <row r="166" spans="1:10" ht="30" x14ac:dyDescent="0.45">
       <c r="A166" t="s">
         <v>163</v>
       </c>
@@ -14615,7 +14617,7 @@
         <v>807</v>
       </c>
     </row>
-    <row r="167" spans="1:10" ht="30" x14ac:dyDescent="0.45">
+    <row r="167" spans="1:10" x14ac:dyDescent="0.45">
       <c r="A167" t="s">
         <v>164</v>
       </c>
@@ -14648,7 +14650,7 @@
         <v>808</v>
       </c>
     </row>
-    <row r="168" spans="1:10" ht="45" x14ac:dyDescent="0.45">
+    <row r="168" spans="1:10" x14ac:dyDescent="0.45">
       <c r="A168" t="s">
         <v>165</v>
       </c>
@@ -14681,7 +14683,7 @@
         <v>809</v>
       </c>
     </row>
-    <row r="169" spans="1:10" ht="60" x14ac:dyDescent="0.45">
+    <row r="169" spans="1:10" x14ac:dyDescent="0.45">
       <c r="A169" t="s">
         <v>166</v>
       </c>
@@ -14714,7 +14716,7 @@
         <v>810</v>
       </c>
     </row>
-    <row r="170" spans="1:10" ht="45" x14ac:dyDescent="0.45">
+    <row r="170" spans="1:10" ht="30" x14ac:dyDescent="0.45">
       <c r="A170" t="s">
         <v>167</v>
       </c>
@@ -14747,7 +14749,7 @@
         <v>811</v>
       </c>
     </row>
-    <row r="171" spans="1:10" ht="45" x14ac:dyDescent="0.45">
+    <row r="171" spans="1:10" x14ac:dyDescent="0.45">
       <c r="A171" t="s">
         <v>168</v>
       </c>
@@ -14780,7 +14782,7 @@
         <v>812</v>
       </c>
     </row>
-    <row r="172" spans="1:10" ht="60" x14ac:dyDescent="0.45">
+    <row r="172" spans="1:10" ht="30" x14ac:dyDescent="0.45">
       <c r="A172" t="s">
         <v>169</v>
       </c>
@@ -14813,7 +14815,7 @@
         <v>813</v>
       </c>
     </row>
-    <row r="173" spans="1:10" ht="45" x14ac:dyDescent="0.45">
+    <row r="173" spans="1:10" ht="30" x14ac:dyDescent="0.45">
       <c r="A173" t="s">
         <v>170</v>
       </c>
@@ -14846,7 +14848,7 @@
         <v>814</v>
       </c>
     </row>
-    <row r="174" spans="1:10" ht="60" x14ac:dyDescent="0.45">
+    <row r="174" spans="1:10" x14ac:dyDescent="0.45">
       <c r="A174" t="s">
         <v>171</v>
       </c>
@@ -14879,7 +14881,7 @@
         <v>815</v>
       </c>
     </row>
-    <row r="175" spans="1:10" ht="60" x14ac:dyDescent="0.45">
+    <row r="175" spans="1:10" ht="30" x14ac:dyDescent="0.45">
       <c r="A175" t="s">
         <v>172</v>
       </c>
@@ -14912,7 +14914,7 @@
         <v>816</v>
       </c>
     </row>
-    <row r="176" spans="1:10" ht="45" x14ac:dyDescent="0.45">
+    <row r="176" spans="1:10" ht="30" x14ac:dyDescent="0.45">
       <c r="A176" t="s">
         <v>173</v>
       </c>
@@ -14945,7 +14947,7 @@
         <v>817</v>
       </c>
     </row>
-    <row r="177" spans="1:10" ht="45" x14ac:dyDescent="0.45">
+    <row r="177" spans="1:10" x14ac:dyDescent="0.45">
       <c r="A177" t="s">
         <v>174</v>
       </c>
@@ -14978,7 +14980,7 @@
         <v>818</v>
       </c>
     </row>
-    <row r="178" spans="1:10" ht="45" x14ac:dyDescent="0.45">
+    <row r="178" spans="1:10" x14ac:dyDescent="0.45">
       <c r="A178" t="s">
         <v>175</v>
       </c>
@@ -15042,7 +15044,7 @@
       </c>
       <c r="J179" s="12"/>
     </row>
-    <row r="180" spans="1:10" ht="45" x14ac:dyDescent="0.45">
+    <row r="180" spans="1:10" ht="30" x14ac:dyDescent="0.45">
       <c r="A180" t="s">
         <v>177</v>
       </c>
@@ -15075,7 +15077,7 @@
         <v>820</v>
       </c>
     </row>
-    <row r="181" spans="1:10" ht="45" x14ac:dyDescent="0.45">
+    <row r="181" spans="1:10" x14ac:dyDescent="0.45">
       <c r="A181" t="s">
         <v>178</v>
       </c>
@@ -15108,7 +15110,7 @@
         <v>821</v>
       </c>
     </row>
-    <row r="182" spans="1:10" ht="60" x14ac:dyDescent="0.45">
+    <row r="182" spans="1:10" ht="30" x14ac:dyDescent="0.45">
       <c r="A182" t="s">
         <v>179</v>
       </c>
@@ -15141,7 +15143,7 @@
         <v>822</v>
       </c>
     </row>
-    <row r="183" spans="1:10" ht="45" x14ac:dyDescent="0.45">
+    <row r="183" spans="1:10" ht="30" x14ac:dyDescent="0.45">
       <c r="A183" t="s">
         <v>180</v>
       </c>
@@ -15174,7 +15176,7 @@
         <v>823</v>
       </c>
     </row>
-    <row r="184" spans="1:10" ht="45" x14ac:dyDescent="0.45">
+    <row r="184" spans="1:10" x14ac:dyDescent="0.45">
       <c r="A184" t="s">
         <v>181</v>
       </c>
@@ -15238,7 +15240,7 @@
       </c>
       <c r="J185" s="12"/>
     </row>
-    <row r="186" spans="1:10" ht="45" x14ac:dyDescent="0.45">
+    <row r="186" spans="1:10" x14ac:dyDescent="0.45">
       <c r="A186" t="s">
         <v>183</v>
       </c>
@@ -15271,7 +15273,7 @@
         <v>825</v>
       </c>
     </row>
-    <row r="187" spans="1:10" ht="75" x14ac:dyDescent="0.45">
+    <row r="187" spans="1:10" ht="30" x14ac:dyDescent="0.45">
       <c r="A187" t="s">
         <v>184</v>
       </c>
@@ -15304,7 +15306,7 @@
         <v>826</v>
       </c>
     </row>
-    <row r="188" spans="1:10" ht="75" x14ac:dyDescent="0.45">
+    <row r="188" spans="1:10" ht="30" x14ac:dyDescent="0.45">
       <c r="A188" t="s">
         <v>185</v>
       </c>
@@ -15337,7 +15339,7 @@
         <v>827</v>
       </c>
     </row>
-    <row r="189" spans="1:10" ht="60" x14ac:dyDescent="0.45">
+    <row r="189" spans="1:10" ht="30" x14ac:dyDescent="0.45">
       <c r="A189" t="s">
         <v>186</v>
       </c>
@@ -15370,7 +15372,7 @@
         <v>828</v>
       </c>
     </row>
-    <row r="190" spans="1:10" ht="45" x14ac:dyDescent="0.45">
+    <row r="190" spans="1:10" x14ac:dyDescent="0.45">
       <c r="A190" t="s">
         <v>187</v>
       </c>
@@ -15403,7 +15405,7 @@
         <v>829</v>
       </c>
     </row>
-    <row r="191" spans="1:10" ht="60" x14ac:dyDescent="0.45">
+    <row r="191" spans="1:10" ht="30" x14ac:dyDescent="0.45">
       <c r="A191" t="s">
         <v>39</v>
       </c>
@@ -15436,7 +15438,7 @@
         <v>692</v>
       </c>
     </row>
-    <row r="192" spans="1:10" ht="60" x14ac:dyDescent="0.45">
+    <row r="192" spans="1:10" ht="30" x14ac:dyDescent="0.45">
       <c r="A192" t="s">
         <v>188</v>
       </c>
@@ -15500,7 +15502,7 @@
       </c>
       <c r="J193" s="12"/>
     </row>
-    <row r="194" spans="1:10" ht="45" x14ac:dyDescent="0.45">
+    <row r="194" spans="1:10" x14ac:dyDescent="0.45">
       <c r="A194" t="s">
         <v>190</v>
       </c>
@@ -15533,7 +15535,7 @@
         <v>830</v>
       </c>
     </row>
-    <row r="195" spans="1:10" ht="90" x14ac:dyDescent="0.45">
+    <row r="195" spans="1:10" ht="30" x14ac:dyDescent="0.45">
       <c r="A195" t="s">
         <v>191</v>
       </c>
@@ -15566,7 +15568,7 @@
         <v>831</v>
       </c>
     </row>
-    <row r="196" spans="1:10" ht="60" x14ac:dyDescent="0.45">
+    <row r="196" spans="1:10" x14ac:dyDescent="0.45">
       <c r="A196" t="s">
         <v>192</v>
       </c>
@@ -15599,7 +15601,7 @@
         <v>832</v>
       </c>
     </row>
-    <row r="197" spans="1:10" ht="60" x14ac:dyDescent="0.45">
+    <row r="197" spans="1:10" ht="30" x14ac:dyDescent="0.45">
       <c r="A197" t="s">
         <v>193</v>
       </c>
@@ -15665,7 +15667,7 @@
         <v>834</v>
       </c>
     </row>
-    <row r="199" spans="1:10" ht="60" x14ac:dyDescent="0.45">
+    <row r="199" spans="1:10" ht="30" x14ac:dyDescent="0.45">
       <c r="A199" t="s">
         <v>195</v>
       </c>
@@ -15698,7 +15700,7 @@
         <v>835</v>
       </c>
     </row>
-    <row r="200" spans="1:10" ht="45" x14ac:dyDescent="0.45">
+    <row r="200" spans="1:10" ht="30" x14ac:dyDescent="0.45">
       <c r="A200" t="s">
         <v>196</v>
       </c>
@@ -15731,7 +15733,7 @@
         <v>836</v>
       </c>
     </row>
-    <row r="201" spans="1:10" ht="60" x14ac:dyDescent="0.45">
+    <row r="201" spans="1:10" ht="30" x14ac:dyDescent="0.45">
       <c r="A201" t="s">
         <v>197</v>
       </c>
@@ -15764,7 +15766,7 @@
         <v>837</v>
       </c>
     </row>
-    <row r="202" spans="1:10" ht="60" x14ac:dyDescent="0.45">
+    <row r="202" spans="1:10" ht="30" x14ac:dyDescent="0.45">
       <c r="A202" t="s">
         <v>198</v>
       </c>
@@ -15828,7 +15830,7 @@
       </c>
       <c r="J203" s="12"/>
     </row>
-    <row r="204" spans="1:10" ht="60" x14ac:dyDescent="0.45">
+    <row r="204" spans="1:10" x14ac:dyDescent="0.45">
       <c r="A204" t="s">
         <v>200</v>
       </c>
@@ -15861,7 +15863,7 @@
         <v>839</v>
       </c>
     </row>
-    <row r="205" spans="1:10" ht="45" x14ac:dyDescent="0.45">
+    <row r="205" spans="1:10" x14ac:dyDescent="0.45">
       <c r="A205" t="s">
         <v>201</v>
       </c>
@@ -15925,7 +15927,7 @@
       </c>
       <c r="J206" s="12"/>
     </row>
-    <row r="207" spans="1:10" ht="45" x14ac:dyDescent="0.45">
+    <row r="207" spans="1:10" ht="30" x14ac:dyDescent="0.45">
       <c r="A207" t="s">
         <v>203</v>
       </c>
@@ -15958,7 +15960,7 @@
         <v>841</v>
       </c>
     </row>
-    <row r="208" spans="1:10" ht="45" x14ac:dyDescent="0.45">
+    <row r="208" spans="1:10" x14ac:dyDescent="0.45">
       <c r="A208" t="s">
         <v>204</v>
       </c>
@@ -15991,7 +15993,7 @@
         <v>842</v>
       </c>
     </row>
-    <row r="209" spans="1:10" ht="30" x14ac:dyDescent="0.45">
+    <row r="209" spans="1:10" x14ac:dyDescent="0.45">
       <c r="A209" t="s">
         <v>205</v>
       </c>
@@ -16024,7 +16026,7 @@
         <v>843</v>
       </c>
     </row>
-    <row r="210" spans="1:10" ht="45" x14ac:dyDescent="0.45">
+    <row r="210" spans="1:10" x14ac:dyDescent="0.45">
       <c r="A210" t="s">
         <v>206</v>
       </c>
@@ -16057,7 +16059,7 @@
         <v>844</v>
       </c>
     </row>
-    <row r="211" spans="1:10" ht="60" x14ac:dyDescent="0.45">
+    <row r="211" spans="1:10" ht="15.75" x14ac:dyDescent="0.45">
       <c r="A211" s="2" t="s">
         <v>452</v>
       </c>
@@ -16154,7 +16156,7 @@
       </c>
       <c r="J213" s="12"/>
     </row>
-    <row r="214" spans="1:10" ht="60" x14ac:dyDescent="0.45">
+    <row r="214" spans="1:10" ht="31.5" x14ac:dyDescent="0.45">
       <c r="A214" s="2" t="s">
         <v>455</v>
       </c>
@@ -16187,7 +16189,7 @@
         <v>847</v>
       </c>
     </row>
-    <row r="215" spans="1:10" ht="45" x14ac:dyDescent="0.45">
+    <row r="215" spans="1:10" ht="15.75" x14ac:dyDescent="0.45">
       <c r="A215" s="2" t="s">
         <v>456</v>
       </c>
@@ -16220,7 +16222,7 @@
         <v>848</v>
       </c>
     </row>
-    <row r="216" spans="1:10" ht="30" x14ac:dyDescent="0.45">
+    <row r="216" spans="1:10" ht="15.75" x14ac:dyDescent="0.45">
       <c r="A216" s="2" t="s">
         <v>457</v>
       </c>
@@ -16253,7 +16255,7 @@
         <v>849</v>
       </c>
     </row>
-    <row r="217" spans="1:10" ht="45" x14ac:dyDescent="0.45">
+    <row r="217" spans="1:10" ht="15.75" x14ac:dyDescent="0.45">
       <c r="A217" s="2" t="s">
         <v>458</v>
       </c>
@@ -16286,7 +16288,7 @@
         <v>850</v>
       </c>
     </row>
-    <row r="218" spans="1:10" ht="60" x14ac:dyDescent="0.45">
+    <row r="218" spans="1:10" ht="15.75" x14ac:dyDescent="0.45">
       <c r="A218" s="2" t="s">
         <v>459</v>
       </c>
@@ -16319,7 +16321,7 @@
         <v>851</v>
       </c>
     </row>
-    <row r="219" spans="1:10" ht="45" x14ac:dyDescent="0.45">
+    <row r="219" spans="1:10" ht="15.75" x14ac:dyDescent="0.45">
       <c r="A219" s="2" t="s">
         <v>460</v>
       </c>
@@ -16352,7 +16354,7 @@
         <v>852</v>
       </c>
     </row>
-    <row r="220" spans="1:10" ht="45" x14ac:dyDescent="0.45">
+    <row r="220" spans="1:10" ht="31.5" x14ac:dyDescent="0.45">
       <c r="A220" s="2" t="s">
         <v>461</v>
       </c>
@@ -16385,7 +16387,7 @@
         <v>853</v>
       </c>
     </row>
-    <row r="221" spans="1:10" ht="30" x14ac:dyDescent="0.45">
+    <row r="221" spans="1:10" ht="15.75" x14ac:dyDescent="0.45">
       <c r="A221" s="2" t="s">
         <v>462</v>
       </c>
@@ -16418,7 +16420,7 @@
         <v>854</v>
       </c>
     </row>
-    <row r="222" spans="1:10" ht="45" x14ac:dyDescent="0.45">
+    <row r="222" spans="1:10" ht="15.75" x14ac:dyDescent="0.45">
       <c r="A222" s="2" t="s">
         <v>463</v>
       </c>
@@ -16451,7 +16453,7 @@
         <v>855</v>
       </c>
     </row>
-    <row r="223" spans="1:10" ht="30" x14ac:dyDescent="0.45">
+    <row r="223" spans="1:10" ht="15.75" x14ac:dyDescent="0.45">
       <c r="A223" s="2" t="s">
         <v>464</v>
       </c>
@@ -16484,7 +16486,7 @@
         <v>856</v>
       </c>
     </row>
-    <row r="224" spans="1:10" ht="60" x14ac:dyDescent="0.45">
+    <row r="224" spans="1:10" ht="15.75" x14ac:dyDescent="0.45">
       <c r="A224" s="2" t="s">
         <v>465</v>
       </c>
@@ -16550,7 +16552,7 @@
         <v>858</v>
       </c>
     </row>
-    <row r="226" spans="1:10" ht="30" x14ac:dyDescent="0.45">
+    <row r="226" spans="1:10" ht="15.75" x14ac:dyDescent="0.45">
       <c r="A226" s="2" t="s">
         <v>467</v>
       </c>
@@ -16583,7 +16585,7 @@
         <v>859</v>
       </c>
     </row>
-    <row r="227" spans="1:10" ht="45" x14ac:dyDescent="0.45">
+    <row r="227" spans="1:10" ht="15.75" x14ac:dyDescent="0.45">
       <c r="A227" s="2" t="s">
         <v>468</v>
       </c>
@@ -16616,7 +16618,7 @@
         <v>860</v>
       </c>
     </row>
-    <row r="228" spans="1:10" ht="45" x14ac:dyDescent="0.45">
+    <row r="228" spans="1:10" ht="15.75" x14ac:dyDescent="0.45">
       <c r="A228" s="2" t="s">
         <v>469</v>
       </c>
@@ -16649,7 +16651,7 @@
         <v>861</v>
       </c>
     </row>
-    <row r="229" spans="1:10" ht="30" x14ac:dyDescent="0.45">
+    <row r="229" spans="1:10" ht="15.75" x14ac:dyDescent="0.45">
       <c r="A229" s="2" t="s">
         <v>470</v>
       </c>
@@ -16682,7 +16684,7 @@
         <v>862</v>
       </c>
     </row>
-    <row r="230" spans="1:10" ht="45" x14ac:dyDescent="0.45">
+    <row r="230" spans="1:10" ht="15.75" x14ac:dyDescent="0.45">
       <c r="A230" s="2" t="s">
         <v>471</v>
       </c>
@@ -16715,7 +16717,7 @@
         <v>863</v>
       </c>
     </row>
-    <row r="231" spans="1:10" ht="75" x14ac:dyDescent="0.45">
+    <row r="231" spans="1:10" ht="15.75" x14ac:dyDescent="0.45">
       <c r="A231" s="2" t="s">
         <v>472</v>
       </c>
@@ -16748,7 +16750,7 @@
         <v>864</v>
       </c>
     </row>
-    <row r="232" spans="1:10" ht="45" x14ac:dyDescent="0.45">
+    <row r="232" spans="1:10" ht="15.75" x14ac:dyDescent="0.45">
       <c r="A232" s="2" t="s">
         <v>473</v>
       </c>
@@ -16781,7 +16783,7 @@
         <v>865</v>
       </c>
     </row>
-    <row r="233" spans="1:10" ht="45" x14ac:dyDescent="0.45">
+    <row r="233" spans="1:10" ht="15.75" x14ac:dyDescent="0.45">
       <c r="A233" s="2" t="s">
         <v>474</v>
       </c>
@@ -16845,7 +16847,7 @@
       </c>
       <c r="J234" s="12"/>
     </row>
-    <row r="235" spans="1:10" ht="60" x14ac:dyDescent="0.45">
+    <row r="235" spans="1:10" ht="15.75" x14ac:dyDescent="0.45">
       <c r="A235" s="2" t="s">
         <v>476</v>
       </c>
@@ -16878,7 +16880,7 @@
         <v>867</v>
       </c>
     </row>
-    <row r="236" spans="1:10" ht="60" x14ac:dyDescent="0.45">
+    <row r="236" spans="1:10" ht="15.75" x14ac:dyDescent="0.45">
       <c r="A236" s="2" t="s">
         <v>477</v>
       </c>
@@ -16911,7 +16913,7 @@
         <v>868</v>
       </c>
     </row>
-    <row r="237" spans="1:10" ht="30" x14ac:dyDescent="0.45">
+    <row r="237" spans="1:10" ht="15.75" x14ac:dyDescent="0.45">
       <c r="A237" s="2" t="s">
         <v>478</v>
       </c>
@@ -17006,7 +17008,7 @@
       </c>
       <c r="J239" s="12"/>
     </row>
-    <row r="240" spans="1:10" ht="60" x14ac:dyDescent="0.45">
+    <row r="240" spans="1:10" ht="30" x14ac:dyDescent="0.45">
       <c r="A240" s="2" t="s">
         <v>481</v>
       </c>
@@ -17039,7 +17041,7 @@
         <v>870</v>
       </c>
     </row>
-    <row r="241" spans="1:10" ht="45" x14ac:dyDescent="0.45">
+    <row r="241" spans="1:10" ht="15.75" x14ac:dyDescent="0.45">
       <c r="A241" s="2" t="s">
         <v>482</v>
       </c>
@@ -17072,7 +17074,7 @@
         <v>871</v>
       </c>
     </row>
-    <row r="242" spans="1:10" ht="45" x14ac:dyDescent="0.45">
+    <row r="242" spans="1:10" ht="15.75" x14ac:dyDescent="0.45">
       <c r="A242" s="2" t="s">
         <v>483</v>
       </c>
@@ -17105,7 +17107,7 @@
         <v>872</v>
       </c>
     </row>
-    <row r="243" spans="1:10" ht="75" x14ac:dyDescent="0.45">
+    <row r="243" spans="1:10" ht="30" x14ac:dyDescent="0.45">
       <c r="A243" s="2" t="s">
         <v>158</v>
       </c>
@@ -17171,7 +17173,7 @@
         <v>873</v>
       </c>
     </row>
-    <row r="245" spans="1:10" ht="60" x14ac:dyDescent="0.45">
+    <row r="245" spans="1:10" ht="30" x14ac:dyDescent="0.45">
       <c r="A245" s="2" t="s">
         <v>485</v>
       </c>
@@ -17204,7 +17206,7 @@
         <v>874</v>
       </c>
     </row>
-    <row r="246" spans="1:10" ht="45" x14ac:dyDescent="0.45">
+    <row r="246" spans="1:10" ht="15.75" x14ac:dyDescent="0.45">
       <c r="A246" s="2" t="s">
         <v>486</v>
       </c>
@@ -17237,7 +17239,7 @@
         <v>875</v>
       </c>
     </row>
-    <row r="247" spans="1:10" ht="45" x14ac:dyDescent="0.45">
+    <row r="247" spans="1:10" ht="15.75" x14ac:dyDescent="0.45">
       <c r="A247" s="2" t="s">
         <v>487</v>
       </c>
@@ -17270,7 +17272,7 @@
         <v>876</v>
       </c>
     </row>
-    <row r="248" spans="1:10" ht="45" x14ac:dyDescent="0.45">
+    <row r="248" spans="1:10" ht="15.75" x14ac:dyDescent="0.45">
       <c r="A248" s="2" t="s">
         <v>488</v>
       </c>
@@ -17303,7 +17305,7 @@
         <v>877</v>
       </c>
     </row>
-    <row r="249" spans="1:10" ht="60" x14ac:dyDescent="0.45">
+    <row r="249" spans="1:10" ht="15.75" x14ac:dyDescent="0.45">
       <c r="A249" s="2" t="s">
         <v>489</v>
       </c>
@@ -17367,7 +17369,7 @@
       </c>
       <c r="J250" s="12"/>
     </row>
-    <row r="251" spans="1:10" ht="75" x14ac:dyDescent="0.45">
+    <row r="251" spans="1:10" ht="31.5" x14ac:dyDescent="0.45">
       <c r="A251" s="2" t="s">
         <v>491</v>
       </c>
@@ -17400,7 +17402,7 @@
         <v>879</v>
       </c>
     </row>
-    <row r="252" spans="1:10" ht="45" x14ac:dyDescent="0.45">
+    <row r="252" spans="1:10" ht="15.75" x14ac:dyDescent="0.45">
       <c r="A252" s="2" t="s">
         <v>492</v>
       </c>
@@ -17433,7 +17435,7 @@
         <v>880</v>
       </c>
     </row>
-    <row r="253" spans="1:10" ht="45" x14ac:dyDescent="0.45">
+    <row r="253" spans="1:10" ht="15.75" x14ac:dyDescent="0.45">
       <c r="A253" s="2" t="s">
         <v>493</v>
       </c>
@@ -17466,7 +17468,7 @@
         <v>881</v>
       </c>
     </row>
-    <row r="254" spans="1:10" ht="45" x14ac:dyDescent="0.45">
+    <row r="254" spans="1:10" ht="15.75" x14ac:dyDescent="0.45">
       <c r="A254" s="2" t="s">
         <v>494</v>
       </c>
@@ -17499,7 +17501,7 @@
         <v>882</v>
       </c>
     </row>
-    <row r="255" spans="1:10" ht="75" x14ac:dyDescent="0.45">
+    <row r="255" spans="1:10" ht="15.75" x14ac:dyDescent="0.45">
       <c r="A255" s="2" t="s">
         <v>495</v>
       </c>
@@ -17532,7 +17534,7 @@
         <v>883</v>
       </c>
     </row>
-    <row r="256" spans="1:10" ht="30" x14ac:dyDescent="0.45">
+    <row r="256" spans="1:10" ht="15.75" x14ac:dyDescent="0.45">
       <c r="A256" s="2" t="s">
         <v>496</v>
       </c>
@@ -17565,7 +17567,7 @@
         <v>884</v>
       </c>
     </row>
-    <row r="257" spans="1:10" ht="60" x14ac:dyDescent="0.45">
+    <row r="257" spans="1:10" ht="30" x14ac:dyDescent="0.45">
       <c r="A257" s="2" t="s">
         <v>497</v>
       </c>
@@ -17598,7 +17600,7 @@
         <v>885</v>
       </c>
     </row>
-    <row r="258" spans="1:10" ht="45" x14ac:dyDescent="0.45">
+    <row r="258" spans="1:10" ht="15.75" x14ac:dyDescent="0.45">
       <c r="A258" s="2" t="s">
         <v>13</v>
       </c>
@@ -17631,7 +17633,7 @@
         <v>667</v>
       </c>
     </row>
-    <row r="259" spans="1:10" ht="45" x14ac:dyDescent="0.45">
+    <row r="259" spans="1:10" ht="15.75" x14ac:dyDescent="0.45">
       <c r="A259" s="2" t="s">
         <v>498</v>
       </c>
@@ -17664,7 +17666,7 @@
         <v>886</v>
       </c>
     </row>
-    <row r="260" spans="1:10" ht="45" x14ac:dyDescent="0.45">
+    <row r="260" spans="1:10" ht="15.75" x14ac:dyDescent="0.45">
       <c r="A260" s="2" t="s">
         <v>499</v>
       </c>
@@ -17728,7 +17730,7 @@
       </c>
       <c r="J261" s="12"/>
     </row>
-    <row r="262" spans="1:10" ht="60" x14ac:dyDescent="0.45">
+    <row r="262" spans="1:10" ht="30" x14ac:dyDescent="0.45">
       <c r="A262" s="2" t="s">
         <v>501</v>
       </c>
@@ -17761,7 +17763,7 @@
         <v>888</v>
       </c>
     </row>
-    <row r="263" spans="1:10" ht="45" x14ac:dyDescent="0.45">
+    <row r="263" spans="1:10" ht="15.75" x14ac:dyDescent="0.45">
       <c r="A263" s="2" t="s">
         <v>502</v>
       </c>
@@ -17794,7 +17796,7 @@
         <v>889</v>
       </c>
     </row>
-    <row r="264" spans="1:10" ht="60" x14ac:dyDescent="0.45">
+    <row r="264" spans="1:10" ht="15.75" x14ac:dyDescent="0.45">
       <c r="A264" s="2" t="s">
         <v>503</v>
       </c>
@@ -17827,7 +17829,7 @@
         <v>890</v>
       </c>
     </row>
-    <row r="265" spans="1:10" ht="45" x14ac:dyDescent="0.45">
+    <row r="265" spans="1:10" ht="15.75" x14ac:dyDescent="0.45">
       <c r="A265" s="2" t="s">
         <v>504</v>
       </c>
@@ -17860,7 +17862,7 @@
         <v>891</v>
       </c>
     </row>
-    <row r="266" spans="1:10" ht="60" x14ac:dyDescent="0.45">
+    <row r="266" spans="1:10" ht="15.75" x14ac:dyDescent="0.45">
       <c r="A266" s="2" t="s">
         <v>505</v>
       </c>
@@ -17893,7 +17895,7 @@
         <v>892</v>
       </c>
     </row>
-    <row r="267" spans="1:10" ht="45" x14ac:dyDescent="0.45">
+    <row r="267" spans="1:10" ht="15.75" x14ac:dyDescent="0.45">
       <c r="A267" s="2" t="s">
         <v>506</v>
       </c>
@@ -17926,7 +17928,7 @@
         <v>893</v>
       </c>
     </row>
-    <row r="268" spans="1:10" ht="45" x14ac:dyDescent="0.45">
+    <row r="268" spans="1:10" ht="15.75" x14ac:dyDescent="0.45">
       <c r="A268" s="2" t="s">
         <v>507</v>
       </c>
@@ -17959,7 +17961,7 @@
         <v>894</v>
       </c>
     </row>
-    <row r="269" spans="1:10" ht="60" x14ac:dyDescent="0.45">
+    <row r="269" spans="1:10" ht="15.75" x14ac:dyDescent="0.45">
       <c r="A269" s="2" t="s">
         <v>508</v>
       </c>
@@ -17992,7 +17994,7 @@
         <v>895</v>
       </c>
     </row>
-    <row r="270" spans="1:10" ht="60" x14ac:dyDescent="0.45">
+    <row r="270" spans="1:10" ht="15.75" x14ac:dyDescent="0.45">
       <c r="A270" s="2" t="s">
         <v>509</v>
       </c>
@@ -18025,7 +18027,7 @@
         <v>896</v>
       </c>
     </row>
-    <row r="271" spans="1:10" ht="45" x14ac:dyDescent="0.45">
+    <row r="271" spans="1:10" ht="15.75" x14ac:dyDescent="0.45">
       <c r="A271" s="2" t="s">
         <v>510</v>
       </c>
@@ -18058,7 +18060,7 @@
         <v>897</v>
       </c>
     </row>
-    <row r="272" spans="1:10" ht="30" x14ac:dyDescent="0.45">
+    <row r="272" spans="1:10" ht="15.75" x14ac:dyDescent="0.45">
       <c r="A272" s="2" t="s">
         <v>41</v>
       </c>
@@ -18091,7 +18093,7 @@
         <v>675</v>
       </c>
     </row>
-    <row r="273" spans="1:10" ht="45" x14ac:dyDescent="0.45">
+    <row r="273" spans="1:10" ht="15.75" x14ac:dyDescent="0.45">
       <c r="A273" s="2" t="s">
         <v>511</v>
       </c>
@@ -18124,7 +18126,7 @@
         <v>898</v>
       </c>
     </row>
-    <row r="274" spans="1:10" ht="60" x14ac:dyDescent="0.45">
+    <row r="274" spans="1:10" ht="30" x14ac:dyDescent="0.45">
       <c r="A274" s="2" t="s">
         <v>512</v>
       </c>
@@ -18157,7 +18159,7 @@
         <v>899</v>
       </c>
     </row>
-    <row r="275" spans="1:10" ht="60" x14ac:dyDescent="0.45">
+    <row r="275" spans="1:10" ht="30" x14ac:dyDescent="0.45">
       <c r="A275" s="2" t="s">
         <v>513</v>
       </c>
@@ -18190,7 +18192,7 @@
         <v>900</v>
       </c>
     </row>
-    <row r="276" spans="1:10" ht="45" x14ac:dyDescent="0.45">
+    <row r="276" spans="1:10" ht="15.75" x14ac:dyDescent="0.45">
       <c r="A276" s="2" t="s">
         <v>514</v>
       </c>
@@ -18223,7 +18225,7 @@
         <v>901</v>
       </c>
     </row>
-    <row r="277" spans="1:10" ht="60" x14ac:dyDescent="0.45">
+    <row r="277" spans="1:10" ht="30" x14ac:dyDescent="0.45">
       <c r="A277" s="2" t="s">
         <v>515</v>
       </c>
@@ -18256,7 +18258,7 @@
         <v>902</v>
       </c>
     </row>
-    <row r="278" spans="1:10" ht="60" x14ac:dyDescent="0.45">
+    <row r="278" spans="1:10" ht="31.5" x14ac:dyDescent="0.45">
       <c r="A278" s="2" t="s">
         <v>516</v>
       </c>
@@ -18289,7 +18291,7 @@
         <v>903</v>
       </c>
     </row>
-    <row r="279" spans="1:10" ht="45" x14ac:dyDescent="0.45">
+    <row r="279" spans="1:10" ht="15.75" x14ac:dyDescent="0.45">
       <c r="A279" s="2" t="s">
         <v>517</v>
       </c>
@@ -18353,7 +18355,7 @@
       </c>
       <c r="J280" s="12"/>
     </row>
-    <row r="281" spans="1:10" ht="45" x14ac:dyDescent="0.45">
+    <row r="281" spans="1:10" ht="15.75" x14ac:dyDescent="0.45">
       <c r="A281" s="2" t="s">
         <v>519</v>
       </c>
@@ -18386,7 +18388,7 @@
         <v>905</v>
       </c>
     </row>
-    <row r="282" spans="1:10" ht="45" x14ac:dyDescent="0.45">
+    <row r="282" spans="1:10" ht="15.75" x14ac:dyDescent="0.45">
       <c r="A282" s="2" t="s">
         <v>520</v>
       </c>
@@ -18419,7 +18421,7 @@
         <v>906</v>
       </c>
     </row>
-    <row r="283" spans="1:10" ht="45" x14ac:dyDescent="0.45">
+    <row r="283" spans="1:10" ht="31.5" x14ac:dyDescent="0.45">
       <c r="A283" s="2" t="s">
         <v>521</v>
       </c>
@@ -18452,7 +18454,7 @@
         <v>907</v>
       </c>
     </row>
-    <row r="284" spans="1:10" ht="45" x14ac:dyDescent="0.45">
+    <row r="284" spans="1:10" ht="30" x14ac:dyDescent="0.45">
       <c r="A284" s="2" t="s">
         <v>522</v>
       </c>
@@ -18516,7 +18518,7 @@
       </c>
       <c r="J285" s="12"/>
     </row>
-    <row r="286" spans="1:10" ht="75" x14ac:dyDescent="0.45">
+    <row r="286" spans="1:10" ht="30" x14ac:dyDescent="0.45">
       <c r="A286" s="2" t="s">
         <v>524</v>
       </c>
@@ -18611,7 +18613,7 @@
       </c>
       <c r="J288" s="12"/>
     </row>
-    <row r="289" spans="1:10" ht="60" x14ac:dyDescent="0.45">
+    <row r="289" spans="1:10" ht="30" x14ac:dyDescent="0.45">
       <c r="A289" s="2" t="s">
         <v>527</v>
       </c>
@@ -18675,7 +18677,7 @@
       </c>
       <c r="J290" s="12"/>
     </row>
-    <row r="291" spans="1:10" ht="60" x14ac:dyDescent="0.45">
+    <row r="291" spans="1:10" ht="30" x14ac:dyDescent="0.45">
       <c r="A291" s="2" t="s">
         <v>529</v>
       </c>
@@ -18708,7 +18710,7 @@
         <v>911</v>
       </c>
     </row>
-    <row r="292" spans="1:10" ht="45" x14ac:dyDescent="0.45">
+    <row r="292" spans="1:10" ht="15.75" x14ac:dyDescent="0.45">
       <c r="A292" s="2" t="s">
         <v>530</v>
       </c>
@@ -18741,7 +18743,7 @@
         <v>912</v>
       </c>
     </row>
-    <row r="293" spans="1:10" ht="30" x14ac:dyDescent="0.45">
+    <row r="293" spans="1:10" ht="15.75" x14ac:dyDescent="0.45">
       <c r="A293" s="2" t="s">
         <v>531</v>
       </c>
@@ -18774,7 +18776,7 @@
         <v>913</v>
       </c>
     </row>
-    <row r="294" spans="1:10" ht="60" x14ac:dyDescent="0.45">
+    <row r="294" spans="1:10" ht="15.75" x14ac:dyDescent="0.45">
       <c r="A294" s="2" t="s">
         <v>532</v>
       </c>
@@ -18807,7 +18809,7 @@
         <v>914</v>
       </c>
     </row>
-    <row r="295" spans="1:10" ht="45" x14ac:dyDescent="0.45">
+    <row r="295" spans="1:10" ht="30" x14ac:dyDescent="0.45">
       <c r="A295" s="2" t="s">
         <v>533</v>
       </c>
@@ -18871,7 +18873,7 @@
       </c>
       <c r="J296" s="12"/>
     </row>
-    <row r="297" spans="1:10" ht="45" x14ac:dyDescent="0.45">
+    <row r="297" spans="1:10" ht="30" x14ac:dyDescent="0.45">
       <c r="A297" s="2" t="s">
         <v>535</v>
       </c>
@@ -18937,7 +18939,7 @@
         <v>917</v>
       </c>
     </row>
-    <row r="299" spans="1:10" ht="45" x14ac:dyDescent="0.45">
+    <row r="299" spans="1:10" ht="30" x14ac:dyDescent="0.45">
       <c r="A299" s="2" t="s">
         <v>537</v>
       </c>
@@ -19001,7 +19003,7 @@
       </c>
       <c r="J300" s="12"/>
     </row>
-    <row r="301" spans="1:10" ht="75" x14ac:dyDescent="0.45">
+    <row r="301" spans="1:10" ht="31.5" x14ac:dyDescent="0.45">
       <c r="A301" s="2" t="s">
         <v>539</v>
       </c>
@@ -19034,7 +19036,7 @@
         <v>919</v>
       </c>
     </row>
-    <row r="302" spans="1:10" ht="45" x14ac:dyDescent="0.45">
+    <row r="302" spans="1:10" ht="31.5" x14ac:dyDescent="0.45">
       <c r="A302" s="3" t="s">
         <v>540</v>
       </c>
@@ -19067,7 +19069,7 @@
         <v>920</v>
       </c>
     </row>
-    <row r="303" spans="1:10" ht="45" x14ac:dyDescent="0.45">
+    <row r="303" spans="1:10" ht="15.75" x14ac:dyDescent="0.45">
       <c r="A303" s="4" t="s">
         <v>541</v>
       </c>
@@ -19100,7 +19102,7 @@
         <v>727</v>
       </c>
     </row>
-    <row r="304" spans="1:10" ht="120" x14ac:dyDescent="0.45">
+    <row r="304" spans="1:10" ht="45" x14ac:dyDescent="0.45">
       <c r="A304" s="4" t="s">
         <v>542</v>
       </c>
@@ -19122,10 +19124,6 @@
       <c r="G304" t="s">
         <v>447</v>
       </c>
-      <c r="H304" s="6">
-        <f>VLOOKUP(A304, '[1]Marini+iDigBio'!$D$2:$J$306, 7, FALSE)</f>
-        <v>0</v>
-      </c>
       <c r="I304" t="e">
         <v>#N/A</v>
       </c>
@@ -19133,7 +19131,7 @@
         <v>921</v>
       </c>
     </row>
-    <row r="305" spans="1:10" ht="60" x14ac:dyDescent="0.45">
+    <row r="305" spans="1:10" ht="30" x14ac:dyDescent="0.45">
       <c r="A305" s="4" t="s">
         <v>543</v>
       </c>
@@ -19155,10 +19153,6 @@
       <c r="G305" t="s">
         <v>447</v>
       </c>
-      <c r="H305" s="6">
-        <f>VLOOKUP(A305, '[1]Marini+iDigBio'!$D$2:$J$306, 7, FALSE)</f>
-        <v>0</v>
-      </c>
       <c r="I305" t="e">
         <v>#N/A</v>
       </c>
@@ -19166,7 +19160,7 @@
         <v>733</v>
       </c>
     </row>
-    <row r="306" spans="1:10" ht="60" x14ac:dyDescent="0.45">
+    <row r="306" spans="1:10" ht="15.75" x14ac:dyDescent="0.45">
       <c r="A306" s="4" t="s">
         <v>544</v>
       </c>
@@ -19187,10 +19181,6 @@
       </c>
       <c r="G306" t="s">
         <v>447</v>
-      </c>
-      <c r="H306" s="6">
-        <f>VLOOKUP(A306, '[1]Marini+iDigBio'!$D$2:$J$306, 7, FALSE)</f>
-        <v>0</v>
       </c>
       <c r="I306" t="e">
         <v>#N/A</v>
@@ -21311,7 +21301,7 @@
       <c r="J1000" s="12"/>
     </row>
   </sheetData>
-  <autoFilter ref="A1:I306" xr:uid="{00000000-0009-0000-0000-000000000000}"/>
+  <autoFilter ref="A1:I307" xr:uid="{00000000-0009-0000-0000-000000000000}"/>
   <phoneticPr fontId="5" type="noConversion"/>
   <hyperlinks>
     <hyperlink ref="J2" r:id="rId1" display="https://www.nhm.ac.uk/" xr:uid="{305EF9E5-9F84-4710-A3B4-BAAF1B556BF1}"/>

</xml_diff>